<commit_message>
feat: compare temporal baselines and support clean handover
</commit_message>
<xml_diff>
--- a/Tho_Churn_Prediction/outputs/temporal_v3_provisional/temporal_summary.xlsx
+++ b/Tho_Churn_Prediction/outputs/temporal_v3_provisional/temporal_summary.xlsx
@@ -11,13 +11,14 @@
     <sheet name="Classification" sheetId="2" r:id="rId2"/>
     <sheet name="Confusion_matrix" sheetId="3" r:id="rId3"/>
     <sheet name="Feature_importance" sheetId="4" r:id="rId4"/>
+    <sheet name="Baseline_comparison" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="68">
   <si>
     <t>Chỉ tiêu</t>
   </si>
@@ -194,6 +195,33 @@
   </si>
   <si>
     <t>category__region_name_Centro-Oeste</t>
+  </si>
+  <si>
+    <t>Mô hình</t>
+  </si>
+  <si>
+    <t>Accuracy</t>
+  </si>
+  <si>
+    <t>Recall mua lại</t>
+  </si>
+  <si>
+    <t>Precision mua lại</t>
+  </si>
+  <si>
+    <t>F1 mua lại</t>
+  </si>
+  <si>
+    <t>ROC-AUC</t>
+  </si>
+  <si>
+    <t>random_forest</t>
+  </si>
+  <si>
+    <t>logistic_regression</t>
+  </si>
+  <si>
+    <t>always_no_repurchase</t>
   </si>
 </sst>
 </file>
@@ -1023,4 +1051,102 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2">
+        <v>0.9491525423728814</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0.6420084635416666</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3">
+        <v>0.6091101694915254</v>
+      </c>
+      <c r="C3">
+        <v>0.5625</v>
+      </c>
+      <c r="D3">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="E3">
+        <v>0.1276595744680851</v>
+      </c>
+      <c r="F3">
+        <v>0.6253720238095238</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4">
+        <v>0.9491525423728814</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>